<commit_message>
4.11.2026 - Update 1
</commit_message>
<xml_diff>
--- a/DATA/MULTI POSITION SPLIT DATA.xlsx
+++ b/DATA/MULTI POSITION SPLIT DATA.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ericc\Documents\HHpro\DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f74da922c65ffa9a/Desktop/HHpro/_TEMP WORK FILES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B210EB-9DB9-4EE5-B5BB-51A01E4269FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{61B210EB-9DB9-4EE5-B5BB-51A01E4269FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FA76716-F3DD-4671-8931-092780C27498}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{52EB5844-5BB7-4D5A-9C1E-11A984DD24F6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{52EB5844-5BB7-4D5A-9C1E-11A984DD24F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Multi Position Splits" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Schedule Notes" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13223" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13227" uniqueCount="310">
   <si>
     <t>MULTI POSITION SPLIT SYSTEM SCHEDULE</t>
   </si>
@@ -956,6 +956,18 @@
   <si>
     <t>19.0 SEER2</t>
   </si>
+  <si>
+    <t>Provide with 7-day programmable thermostat</t>
+  </si>
+  <si>
+    <t>Provide with 7-day programmable BACnet thermostat</t>
+  </si>
+  <si>
+    <t>Provide with field installed disconnect. Disconnect shall be provided and installed by electrical contractor</t>
+  </si>
+  <si>
+    <t>Electric heat, if scheduled, shall be single point power.  kW listed is at 240V &amp; temperature rise has 0.75 multiplier applied for 230V</t>
+  </si>
 </sst>
 </file>
 
@@ -1635,30 +1647,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1681,6 +1669,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1694,6 +1688,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2078,38 +2090,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="51"/>
-      <c r="Y1" s="51"/>
-      <c r="Z1" s="51"/>
-      <c r="AA1" s="51"/>
-      <c r="AB1" s="51"/>
-      <c r="AC1" s="51"/>
-      <c r="AD1" s="52"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
+      <c r="AD1" s="44"/>
       <c r="AE1" s="33" t="s">
         <v>1</v>
       </c>
@@ -2149,13 +2161,13 @@
       <c r="AB2" s="31"/>
       <c r="AC2" s="31"/>
       <c r="AD2" s="32"/>
-      <c r="AE2" s="53"/>
+      <c r="AE2" s="45"/>
     </row>
     <row r="3" spans="1:53" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="48" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -2163,13 +2175,13 @@
       </c>
       <c r="D3" s="31"/>
       <c r="E3" s="32"/>
-      <c r="F3" s="56" t="s">
+      <c r="F3" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="58"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="52"/>
       <c r="K3" s="33" t="s">
         <v>8</v>
       </c>
@@ -2177,30 +2189,30 @@
         <v>9</v>
       </c>
       <c r="M3" s="32"/>
-      <c r="N3" s="39" t="s">
+      <c r="N3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="40"/>
-      <c r="P3" s="41"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="55"/>
       <c r="Q3" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="R3" s="42" t="s">
+      <c r="R3" s="46" t="s">
         <v>4</v>
       </c>
       <c r="S3" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="T3" s="44" t="s">
+      <c r="T3" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="U3" s="45"/>
-      <c r="V3" s="46"/>
-      <c r="W3" s="47" t="s">
+      <c r="U3" s="57"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="X3" s="48"/>
-      <c r="Y3" s="49"/>
+      <c r="X3" s="40"/>
+      <c r="Y3" s="41"/>
       <c r="Z3" s="33" t="s">
         <v>13</v>
       </c>
@@ -2216,7 +2228,7 @@
       <c r="AD3" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="AE3" s="53"/>
+      <c r="AE3" s="45"/>
       <c r="AG3" s="30" t="s">
         <v>175</v>
       </c>
@@ -2243,8 +2255,8 @@
       <c r="BA3" s="32"/>
     </row>
     <row r="4" spans="1:53" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="43"/>
-      <c r="B4" s="55"/>
+      <c r="A4" s="47"/>
+      <c r="B4" s="49"/>
       <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
@@ -2286,7 +2298,7 @@
         <v>29</v>
       </c>
       <c r="Q4" s="36"/>
-      <c r="R4" s="43"/>
+      <c r="R4" s="47"/>
       <c r="S4" s="34"/>
       <c r="T4" s="2" t="s">
         <v>30</v>
@@ -81673,9 +81685,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A91E718E-D388-4692-8CAD-841447CEA197}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>